<commit_message>
docs: record final local verification run
</commit_message>
<xml_diff>
--- a/outputs/01a08aec-efc7-7340-b823-2e03084046dd/plandosee-test-evidence.xlsx
+++ b/outputs/01a08aec-efc7-7340-b823-2e03084046dd/plandosee-test-evidence.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R984df274859946ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="테스트 케이스" sheetId="2" r:id="R76b369108deb42f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요구사항 추적" sheetId="3" r:id="R486d30f996374121"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실행 이력" sheetId="4" r:id="Rd116228a84944348"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R7cb977d85a204248"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="테스트 케이스" sheetId="2" r:id="R6a7edfb6fa8f493c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요구사항 추적" sheetId="3" r:id="Red0076457d274cf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실행 이력" sheetId="4" r:id="R31128452333e456d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -628,7 +628,7 @@
         <x:v>로컬</x:v>
       </x:c>
       <x:c r="B13" s="19" t="str">
-        <x:v>2026-09-10 22:35 KST</x:v>
+        <x:v>2026-09-10 23:00 KST</x:v>
       </x:c>
       <x:c r="C13" s="19" t="str">
         <x:v>pnpm test:all</x:v>
@@ -2119,25 +2119,94 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
-      <x:c r="A9" s="21" t="n">
+      <x:c r="A9" s="20" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B9" s="21" t="str">
+      <x:c r="B9" s="20" t="str">
+        <x:v>2026-09-10 22:55</x:v>
+      </x:c>
+      <x:c r="C9" s="20" t="str">
+        <x:v>로컬</x:v>
+      </x:c>
+      <x:c r="D9" s="28" t="str">
+        <x:v>pnpm test:all</x:v>
+      </x:c>
+      <x:c r="E9" s="28" t="str">
+        <x:v>실패</x:v>
+      </x:c>
+      <x:c r="F9" s="28" t="str">
+        <x:v>Codex 작업 종료와 함께 분리 실행한 로컬 DB 프로세스 종료</x:v>
+      </x:c>
+      <x:c r="G9" s="28" t="str">
+        <x:v>DB를 독립 전경 세션으로 재기동</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="A10" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B10" s="20" t="str">
+        <x:v>2026-09-10 22:57</x:v>
+      </x:c>
+      <x:c r="C10" s="20" t="str">
+        <x:v>로컬</x:v>
+      </x:c>
+      <x:c r="D10" s="28" t="str">
+        <x:v>pnpm test:all</x:v>
+      </x:c>
+      <x:c r="E10" s="28" t="str">
+        <x:v>실패</x:v>
+      </x:c>
+      <x:c r="F10" s="28" t="str">
+        <x:v>동일 환경 수명 문제 재현</x:v>
+      </x:c>
+      <x:c r="G10" s="28" t="str">
+        <x:v>새 로컬 DB 생성·마이그레이션·시드</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="34" customHeight="1">
+      <x:c r="A11" s="20" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B11" s="20" t="str">
+        <x:v>2026-09-10 23:00</x:v>
+      </x:c>
+      <x:c r="C11" s="20" t="str">
+        <x:v>로컬</x:v>
+      </x:c>
+      <x:c r="D11" s="28" t="str">
+        <x:v>pnpm test:all</x:v>
+      </x:c>
+      <x:c r="E11" s="28" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="F11" s="28" t="str">
+        <x:v>단위 8·E2E 6, 린트·타입·빌드 통과</x:v>
+      </x:c>
+      <x:c r="G11" s="28" t="str">
+        <x:v>최종 로컬 기준선 확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="34" customHeight="1">
+      <x:c r="A12" s="21" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B12" s="21" t="str">
         <x:v>배포 후</x:v>
       </x:c>
-      <x:c r="C9" s="21" t="str">
+      <x:c r="C12" s="21" t="str">
         <x:v>운영</x:v>
       </x:c>
-      <x:c r="D9" s="29" t="str">
+      <x:c r="D12" s="29" t="str">
         <x:v>pnpm test:e2e:production</x:v>
       </x:c>
-      <x:c r="E9" s="29" t="str">
+      <x:c r="E12" s="29" t="str">
         <x:v>대기</x:v>
       </x:c>
-      <x:c r="F9" s="29" t="str">
+      <x:c r="F12" s="29" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="G9" s="29" t="str">
+      <x:c r="G12" s="29" t="str">
         <x:v>운영 URL 확정 후 실행</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
test: verify production deployment and record evidence
</commit_message>
<xml_diff>
--- a/outputs/01a08aec-efc7-7340-b823-2e03084046dd/plandosee-test-evidence.xlsx
+++ b/outputs/01a08aec-efc7-7340-b823-2e03084046dd/plandosee-test-evidence.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R7cb977d85a204248"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="테스트 케이스" sheetId="2" r:id="R6a7edfb6fa8f493c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요구사항 추적" sheetId="3" r:id="Red0076457d274cf6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실행 이력" sheetId="4" r:id="R31128452333e456d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R73ce85640eaa4bd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="테스트 케이스" sheetId="2" r:id="R232f75913e0f4bd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요구사항 추적" sheetId="3" r:id="Rb33f07ba91b74d9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실행 이력" sheetId="4" r:id="R28036c4d5225413e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -133,7 +133,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="32">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -219,6 +219,10 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -231,7 +235,7 @@
         <x:color rgb="FF237A57"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5F6EC"/>
         </x:patternFill>
       </x:fill>
@@ -242,7 +246,7 @@
         <x:color rgb="FF9A6700"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -483,7 +487,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>로컬 및 운영 검증 결과 · Asia/Seoul · 2026-09-10</x:v>
+        <x:v>로컬 및 운영 검증 결과 · Asia/Seoul · 2026-09-11</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -548,7 +552,7 @@
       </x:c>
       <x:c r="B8" s="15" t="n">
         <x:f>COUNTIF('테스트 케이스'!$H$7:$H$200,"통과")</x:f>
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C8" s="2"/>
       <x:c r="D8" s="2"/>
@@ -578,7 +582,7 @@
       </x:c>
       <x:c r="B10" s="15" t="n">
         <x:f>COUNTIF('테스트 케이스'!$H$7:$H$200,"대기")</x:f>
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C10" s="2"/>
       <x:c r="D10" s="2"/>
@@ -654,25 +658,25 @@
         <x:v>운영</x:v>
       </x:c>
       <x:c r="B14" s="20" t="str">
-        <x:v>배포 후 갱신</x:v>
+        <x:v>2026-09-11 09:32 KST</x:v>
       </x:c>
       <x:c r="C14" s="20" t="str">
-        <x:v>Vercel URL</x:v>
+        <x:v>https://plandosee-chi.vercel.app</x:v>
       </x:c>
       <x:c r="D14" s="20" t="str">
-        <x:v>익명 스모크</x:v>
+        <x:v>4 E2E</x:v>
       </x:c>
       <x:c r="E14" s="20" t="str">
         <x:v>Chromium</x:v>
       </x:c>
       <x:c r="F14" s="20" t="str">
-        <x:v>대기</x:v>
+        <x:v>모두 통과</x:v>
       </x:c>
       <x:c r="G14" s="20" t="n">
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H14" s="20" t="str">
-        <x:v>시크릿 컨텍스트</x:v>
+        <x:v>익명·DB·복원·보안</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -748,11 +752,11 @@
       <x:c r="H19" s="26"/>
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
-      <x:c r="A20" s="25" t="str">
-        <x:v>운영 대기</x:v>
+      <x:c r="A20" s="24" t="str">
+        <x:v>운영 통과</x:v>
       </x:c>
       <x:c r="B20" s="26" t="str">
-        <x:v>Vercel 배포와 익명 운영 검증 후 동일 파일을 갱신합니다.</x:v>
+        <x:v>Vercel 익명 URL에서 실데이터·집계·복원·내보내기·보안 검증 4건이 모두 통과했습니다.</x:v>
       </x:c>
       <x:c r="C20" s="26"/>
       <x:c r="D20" s="26"/>
@@ -1189,13 +1193,13 @@
         <x:v>인증 없이 표시</x:v>
       </x:c>
       <x:c r="G17" s="28" t="str">
-        <x:v>미실행</x:v>
+        <x:v>익명 표시·모바일·axe 심각 위반 0</x:v>
       </x:c>
       <x:c r="H17" s="20" t="str">
-        <x:v>대기</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="I17" s="20" t="str">
-        <x:v>운영 배포 후 갱신</x:v>
+        <x:v>Playwright JSON</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="32" customHeight="1">
@@ -1218,13 +1222,13 @@
         <x:v>실제 계획 1·할 일 5·기록 3+</x:v>
       </x:c>
       <x:c r="G18" s="28" t="str">
-        <x:v>미실행</x:v>
+        <x:v>계획 1·할 일 7·실행 기록 3, 집계 근거 일치</x:v>
       </x:c>
       <x:c r="H18" s="20" t="str">
-        <x:v>대기</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="I18" s="20" t="str">
-        <x:v>운영 배포 후 갱신</x:v>
+        <x:v>Playwright JSON</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="32" customHeight="1">
@@ -1247,13 +1251,13 @@
         <x:v>자료 유지·JSON 정상</x:v>
       </x:c>
       <x:c r="G19" s="28" t="str">
-        <x:v>미실행</x:v>
+        <x:v>ID·날짜·초 단위·JSON 보존</x:v>
       </x:c>
       <x:c r="H19" s="20" t="str">
-        <x:v>대기</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="I19" s="20" t="str">
-        <x:v>운영 배포 후 갱신</x:v>
+        <x:v>Playwright JSON</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="32" customHeight="1">
@@ -1276,13 +1280,13 @@
         <x:v>비밀 노출 0</x:v>
       </x:c>
       <x:c r="G20" s="29" t="str">
-        <x:v>미실행</x:v>
+        <x:v>비밀 노출 0·콘솔 오류 0</x:v>
       </x:c>
       <x:c r="H20" s="21" t="str">
-        <x:v>대기</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="I20" s="21" t="str">
-        <x:v>운영 배포 후 갱신</x:v>
+        <x:v>Playwright JSON</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1773,7 +1777,7 @@
         <x:v>L-006, P-002</x:v>
       </x:c>
       <x:c r="C36" s="20" t="str">
-        <x:v>로컬 통과·운영 대기</x:v>
+        <x:v>로컬·운영 통과</x:v>
       </x:c>
       <x:c r="D36" s="20" t="str">
         <x:v>docs/REQUIREMENTS.md</x:v>
@@ -1829,7 +1833,7 @@
         <x:v>L-005, L-006, P-002</x:v>
       </x:c>
       <x:c r="C40" s="20" t="str">
-        <x:v>로컬 통과·운영 대기</x:v>
+        <x:v>로컬·운영 통과</x:v>
       </x:c>
       <x:c r="D40" s="20" t="str">
         <x:v>docs/REQUIREMENTS.md</x:v>
@@ -1843,7 +1847,7 @@
         <x:v>L-005, L-006, P-002</x:v>
       </x:c>
       <x:c r="C41" s="20" t="str">
-        <x:v>로컬 통과·운영 대기</x:v>
+        <x:v>로컬·운영 통과</x:v>
       </x:c>
       <x:c r="D41" s="20" t="str">
         <x:v>docs/REQUIREMENTS.md</x:v>
@@ -1857,7 +1861,7 @@
         <x:v>L-005, L-006, P-002</x:v>
       </x:c>
       <x:c r="C42" s="20" t="str">
-        <x:v>로컬 통과·운영 대기</x:v>
+        <x:v>로컬·운영 통과</x:v>
       </x:c>
       <x:c r="D42" s="20" t="str">
         <x:v>docs/REQUIREMENTS.md</x:v>
@@ -1871,7 +1875,7 @@
         <x:v>L-005, L-006, P-002</x:v>
       </x:c>
       <x:c r="C43" s="20" t="str">
-        <x:v>로컬 통과·운영 대기</x:v>
+        <x:v>로컬·운영 통과</x:v>
       </x:c>
       <x:c r="D43" s="20" t="str">
         <x:v>docs/REQUIREMENTS.md</x:v>
@@ -1899,7 +1903,7 @@
         <x:v>L-005, P-001</x:v>
       </x:c>
       <x:c r="C45" s="20" t="str">
-        <x:v>로컬 통과·운영 대기</x:v>
+        <x:v>로컬·운영 통과</x:v>
       </x:c>
       <x:c r="D45" s="20" t="str">
         <x:v>docs/REQUIREMENTS.md</x:v>
@@ -1913,7 +1917,7 @@
         <x:v>L-001, L-004, P-004</x:v>
       </x:c>
       <x:c r="C46" s="20" t="str">
-        <x:v>로컬 통과·운영 대기</x:v>
+        <x:v>로컬·운영 통과</x:v>
       </x:c>
       <x:c r="D46" s="20" t="str">
         <x:v>docs/REQUIREMENTS.md</x:v>
@@ -1969,7 +1973,7 @@
         <x:v>P-001, P-004</x:v>
       </x:c>
       <x:c r="C50" s="21" t="str">
-        <x:v>로컬 통과·운영 대기</x:v>
+        <x:v>로컬·운영 통과</x:v>
       </x:c>
       <x:c r="D50" s="21" t="str">
         <x:v>docs/REQUIREMENTS.md</x:v>
@@ -2188,26 +2192,49 @@
       </x:c>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
-      <x:c r="A12" s="21" t="n">
+      <x:c r="A12" s="20" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B12" s="21" t="str">
-        <x:v>배포 후</x:v>
-      </x:c>
-      <x:c r="C12" s="21" t="str">
+      <x:c r="B12" s="20" t="str">
+        <x:v>2026-09-11 09:27</x:v>
+      </x:c>
+      <x:c r="C12" s="20" t="str">
         <x:v>운영</x:v>
       </x:c>
-      <x:c r="D12" s="29" t="str">
+      <x:c r="D12" s="28" t="str">
         <x:v>pnpm test:e2e:production</x:v>
       </x:c>
-      <x:c r="E12" s="29" t="str">
-        <x:v>대기</x:v>
-      </x:c>
-      <x:c r="F12" s="29" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="G12" s="29" t="str">
-        <x:v>운영 URL 확정 후 실행</x:v>
+      <x:c r="E12" s="28" t="str">
+        <x:v>실패</x:v>
+      </x:c>
+      <x:c r="F12" s="28" t="str">
+        <x:v>화면 locator·비동기 대기·내보내기 필드 경로 불일치</x:v>
+      </x:c>
+      <x:c r="G12" s="28" t="str">
+        <x:v>검증 코드 3건 수정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="34" customHeight="1">
+      <x:c r="A13" s="30" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="str">
+        <x:v>2026-09-11 09:32</x:v>
+      </x:c>
+      <x:c r="C13" s="30" t="str">
+        <x:v>운영</x:v>
+      </x:c>
+      <x:c r="D13" s="31" t="str">
+        <x:v>pnpm test:e2e:production</x:v>
+      </x:c>
+      <x:c r="E13" s="31" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="F13" s="31" t="str">
+        <x:v>운영 E2E 4건 통과</x:v>
+      </x:c>
+      <x:c r="G13" s="31" t="str">
+        <x:v>운영 기준선 확정</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: finalize deployment verification evidence
</commit_message>
<xml_diff>
--- a/outputs/01a08aec-efc7-7340-b823-2e03084046dd/plandosee-test-evidence.xlsx
+++ b/outputs/01a08aec-efc7-7340-b823-2e03084046dd/plandosee-test-evidence.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R73ce85640eaa4bd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="테스트 케이스" sheetId="2" r:id="R232f75913e0f4bd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요구사항 추적" sheetId="3" r:id="Rb33f07ba91b74d9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실행 이력" sheetId="4" r:id="R28036c4d5225413e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R4df1643e16a14aea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="테스트 케이스" sheetId="2" r:id="R5d1288808e6a49d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요구사항 추적" sheetId="3" r:id="R122f1cd54e5e4dae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실행 이력" sheetId="4" r:id="R6096cdd29f744196"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -133,7 +133,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="32">
+  <x:cellXfs count="34">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -222,6 +222,10 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -658,7 +662,7 @@
         <x:v>운영</x:v>
       </x:c>
       <x:c r="B14" s="20" t="str">
-        <x:v>2026-09-11 09:32 KST</x:v>
+        <x:v>2026-09-11 09:44 KST</x:v>
       </x:c>
       <x:c r="C14" s="20" t="str">
         <x:v>https://plandosee-chi.vercel.app</x:v>
@@ -2215,26 +2219,118 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
-      <x:c r="A13" s="30" t="n">
+      <x:c r="A13" s="32" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B13" s="30" t="str">
+      <x:c r="B13" s="32" t="str">
         <x:v>2026-09-11 09:32</x:v>
       </x:c>
-      <x:c r="C13" s="30" t="str">
+      <x:c r="C13" s="32" t="str">
         <x:v>운영</x:v>
       </x:c>
-      <x:c r="D13" s="31" t="str">
+      <x:c r="D13" s="33" t="str">
         <x:v>pnpm test:e2e:production</x:v>
       </x:c>
-      <x:c r="E13" s="31" t="str">
+      <x:c r="E13" s="33" t="str">
         <x:v>통과</x:v>
       </x:c>
-      <x:c r="F13" s="31" t="str">
+      <x:c r="F13" s="33" t="str">
         <x:v>운영 E2E 4건 통과</x:v>
       </x:c>
-      <x:c r="G13" s="31" t="str">
+      <x:c r="G13" s="33" t="str">
         <x:v>운영 기준선 확정</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="34" customHeight="1">
+      <x:c r="A14" s="32" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B14" s="32" t="str">
+        <x:v>2026-09-11 09:40</x:v>
+      </x:c>
+      <x:c r="C14" s="32" t="str">
+        <x:v>운영</x:v>
+      </x:c>
+      <x:c r="D14" s="33" t="str">
+        <x:v>Vercel Git 자동 배포</x:v>
+      </x:c>
+      <x:c r="E14" s="33" t="str">
+        <x:v>실패</x:v>
+      </x:c>
+      <x:c r="F14" s="33" t="str">
+        <x:v>깨끗한 체크아웃에 Prisma 생성 클라이언트 없음</x:v>
+      </x:c>
+      <x:c r="G14" s="33" t="str">
+        <x:v>빌드 앞에 prisma generate 추가</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="32" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B15" s="32" t="str">
+        <x:v>2026-09-11 09:42</x:v>
+      </x:c>
+      <x:c r="C15" s="32" t="str">
+        <x:v>로컬</x:v>
+      </x:c>
+      <x:c r="D15" s="33" t="str">
+        <x:v>pnpm build</x:v>
+      </x:c>
+      <x:c r="E15" s="33" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="F15" s="33" t="str">
+        <x:v>Prisma 생성 후 Next.js 프로덕션 빌드 성공</x:v>
+      </x:c>
+      <x:c r="G15" s="33" t="str">
+        <x:v>clean-build 수정 검증</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="34" customHeight="1">
+      <x:c r="A16" s="32" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B16" s="32" t="str">
+        <x:v>2026-09-11 09:43</x:v>
+      </x:c>
+      <x:c r="C16" s="32" t="str">
+        <x:v>운영</x:v>
+      </x:c>
+      <x:c r="D16" s="33" t="str">
+        <x:v>Vercel Git 자동 배포</x:v>
+      </x:c>
+      <x:c r="E16" s="33" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="F16" s="33" t="str">
+        <x:v>GitHub main 커밋 자동 배포 READY</x:v>
+      </x:c>
+      <x:c r="G16" s="33" t="str">
+        <x:v>공개 별칭 최신화</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="34" customHeight="1">
+      <x:c r="A17" s="32" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B17" s="32" t="str">
+        <x:v>2026-09-11 09:44</x:v>
+      </x:c>
+      <x:c r="C17" s="32" t="str">
+        <x:v>운영</x:v>
+      </x:c>
+      <x:c r="D17" s="33" t="str">
+        <x:v>pnpm test:e2e:production</x:v>
+      </x:c>
+      <x:c r="E17" s="33" t="str">
+        <x:v>통과</x:v>
+      </x:c>
+      <x:c r="F17" s="33" t="str">
+        <x:v>최신 자동 배포에서 E2E 4건 통과</x:v>
+      </x:c>
+      <x:c r="G17" s="33" t="str">
+        <x:v>최종 운영 기준선 확정</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>